<commit_message>
Add MIT license and NuGet package metadata
Adds a LICENSE file and fills in the library's PackageId-adjacent metadata
(version, authors, description, tags, license expression, embedded
README/LICENSE) so it's ready to publish and discoverable by both search and
AI-agent tooling. RepositoryUrl/PackageProjectUrl left unset until there's a
public remote to point at.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
+++ b/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re76bc7772ca54414"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rfa9efff397534a2a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0e00fd75486040fd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6a328bcedb054f28"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -165,7 +165,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rea15b339d06944e0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb91618e2852d44bf"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -213,6 +213,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80235b04453a4edb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1282cfc5f76643c8"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Kookerella.FsOpenXmlDsl.Mcp: an MCP server for the library
A local (stdio) MCP server, distributed as a dotnet tool, exposing three
tools over the core library: create_workbook, read_workbook, and
generate_fsharp_script. Deliberately narrow scope for this first pass (plain
cell values/formulas via a row/column grid, no styling/tables/charts/pivot
tables) - a caller wanting the richer feature set should reference the
library directly.

Input/output DTOs are plain mutable classes rather than F# records, since
System.Text.Json's default reflection deserializer can't construct an
F# record's single all-fields constructor without extra attributes.

Verified by hand-driving the JSON-RPC stdio protocol against the built
executable (initialize / tools/list / tools/call for all three tools,
including a create -> read round trip) and schema-validating the resulting
.xlsx with OpenXmlValidator.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
+++ b/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rfa9efff397534a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R029af13abd8b4507"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6a328bcedb054f28"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra05e100032984c31"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -165,7 +165,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb91618e2852d44bf"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb7317208c57e4b02"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -213,6 +213,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1282cfc5f76643c8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf45d2febdc2e418f"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish Kookerella.FsOpenXmlDsl.Mcp to the official MCP Registry
Adds .mcp/server.json (validated against the live registry schema) and the
required <!-- mcp-name --> README ownership marker, bumping to 0.1.2 since
the marker has to be present in an already-published NuGet README for the
registry to verify it.

Ended up publishing under io.github.MarkNicholls/fsopenxmldsl-mcp rather
than the Kookerella-Ltd org namespace - GitHub org membership visibility
and OAuth app restrictions were both confirmed fine via the API, but the
registry (still an unreleased v0.1 preview) kept rejecting the org
namespace anyway, likely an org-verification gap in the preview registry
rather than anything fixable on the GitHub side. Can revisit once the
registry's org support matures.

Now live: https://registry.modelcontextprotocol.io, listing
io.github.MarkNicholls/fsopenxmldsl-mcp v0.1.2.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
+++ b/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R029af13abd8b4507"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7afb78365b8c416e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra05e100032984c31"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R675fc22cdca1448d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -165,7 +165,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb7317208c57e4b02"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra588d22a7da44d67"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -213,6 +213,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf45d2febdc2e418f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dbb45ccf3d54afe"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add VBA support to the C# wrapper
Workbook.VbaProject (byte[]?) + Workbook.WithVbaProject(byte[]) - opaque
bytes only, same treatment as the F# core's Workbook.VbaProject: no parsing,
generation, or editing of VBA source anywhere in this stack.

One documented exception to "pure everywhere": arrays are reference types,
so WithVbaProject defensively copies its input rather than let a caller
mutate the workbook's bytes after the fact through their original array
reference.

Test project now links (not copies) the F# suite's own sample.vbaProject.bin
- one real fixture extracted from an actual Excel save, shared rather than
duplicated. 3 new tests (12 total): a genuine save/load round trip through
.xlsm with schema validation, the defensive-copy behavior, and the
no-project default case.

Updated the wrapper's README and llms.txt, including a line in llms.txt
that had gone stale (claimed VBA wasn't in the C# wrapper "at all yet").

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
+++ b/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb6bf5420ce0c46b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R86b26d7664e64cae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R178b5ff0c2c944e1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R06825ab098c54133"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -165,7 +165,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf5a0c65863504131"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R70ca5c5b6ca945a7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -213,6 +213,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b82f663b0654f40"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb4002d4870549ed"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Excel Tables to the C# wrapper
TableColumn, TableStyle, TableEntry mirroring the F# core exactly, plus
Sheet.WithTables/AddTable. Reconstructs the F# Worksheet's Tables field the
same way merged ranges/freeze panes/autofilter already do - baseline via
sheetOfCells, override just the fields this wrapper models.

3 new tests (15 total): a basic table, one with a calculated column and
custom style (mirroring the F# suite's own two table scenarios), and a test
confirming the F# core's own validation - column count must match the
range width, column names must be unique - propagates through the wrapper
as ArgumentException with no duplicate validation logic on the C# side.

Updated the wrapper's README (with the validation-error behavior called
out) and llms.txt.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
+++ b/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R86b26d7664e64cae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5f1ae80b4ed64497"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R06825ab098c54133"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5807d907fec54e33"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -165,7 +165,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R70ca5c5b6ca945a7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R45462562f4bf43d5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -213,6 +213,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb4002d4870549ed"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48d39c58aae34e68"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add charts to the C# wrapper
ChartType, ChartSeries, ChartEntry mirroring the F# core exactly, plus
Sheet.WithCharts/AddChart. Reconstructs the F# Worksheet's Charts field the
same way merged ranges/freeze panes/autofilter/tables already do - baseline
via sheetOfCells, override just the fields this wrapper models.

3 new tests (18 total): a column chart with title/legend/two series and a
bar chart without either (mirroring the F# suite's own two chart scenarios),
plus a default-empty/immutability test.

Updated the wrapper's README (with a chart example) and llms.txt.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
+++ b/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5f1ae80b4ed64497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R65d17c56ff124d5e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5807d907fec54e33"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3896d72cb1d54bdf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -165,7 +165,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R45462562f4bf43d5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd55da1d776894d14"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -213,6 +213,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48d39c58aae34e68"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e47b6b085d94665"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add images to the C# wrapper
ImageFormat, ImageEntry mirroring the F# core exactly, plus
Sheet.WithImages/AddImage. Reconstructs the F# Worksheet's Images field the
same way charts/tables/merged ranges/freeze panes/autofilter already do -
baseline via sheetOfCells, override just the fields this wrapper models.

ImageEntry's constructor defensively copies its byte[] Data, same treatment
as Workbook.WithVbaProject and for the same reason - documented on the type.

3 new tests (21 total): a byte-for-byte round trip of the F# suite's own
"1x1 transparent GIF" fixture, a defensive-copy test, and a
default-empty/immutability test.

Updated the wrapper's README (with an image example) and llms.txt.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
+++ b/tests/Kookerella.FsOpenXmlDsl.Tests/Examples/ChartAndImage/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R65d17c56ff124d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R98f8909fcc2849a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3896d72cb1d54bdf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdb8545501db84f37"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -165,7 +165,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd55da1d776894d14"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd308e7f6cf8542c9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -213,6 +213,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e47b6b085d94665"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1607d72ffe714092"/>
 </x:worksheet>
 </file>
</xml_diff>